<commit_message>
reverse engineer excel into DSL
</commit_message>
<xml_diff>
--- a/tests/SafeOpenXml.Tests/Examples/Comments/output.xlsx
+++ b/tests/SafeOpenXml.Tests/Examples/Comments/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R83e0d36995e44c99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc9913622bb1a491a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -92,6 +92,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra73f3b25642f4a19"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bf40c22e4f34ab5"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add print settings and page setup
Adds PageSetup (orientation, paper size, scaling, margins, header/footer)
as a new SheetItem/Worksheet concept, modeled 1:1 on OOXML's
pageMargins/pageSetup/headerFooter elements, including the sheetPr
fitToPage flag that governs whether Excel honors scale% or
fitToWidth/fitToHeight. Wired through Writer, Reader, and CodeGen, with
two new example scenarios verified via schema validation, exact
round-trip, and (in the slow suite) actual dotnet fsi execution of the
generated script.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/SafeOpenXml.Tests/Examples/Comments/output.xlsx
+++ b/tests/SafeOpenXml.Tests/Examples/Comments/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R3607d6891ab14354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R73fdf95da1674a8b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -92,6 +92,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fafcfce8cf446ee"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab42f68820c144ca"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add print area and header/footer variants
Closes both PageSetup gaps: PrintArea (a list of ranges, since Excel
supports several disjoint print rectangles per sheet) transparently
translates to/from OOXML's reserved, hidden, sheet-scoped
_xlnm.Print_Area defined name - the same localSheetId translation
DefinedNameScope.SheetScope already does - so callers never touch
defined names directly. EvenHeader/EvenFooter/FirstHeader/FirstFooter
round out the header/footer model, with Writer automatically setting
the sibling differentOddEven/differentFirst flags whenever they're used.

Two new example scenarios (multi-range print area, first-page/even-page
header/footer) verified via schema validation, exact round-trip, and
(slow suite) actual dotnet fsi execution of the generated script.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/SafeOpenXml.Tests/Examples/Comments/output.xlsx
+++ b/tests/SafeOpenXml.Tests/Examples/Comments/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rfba4ee10952944a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R045858f1a8574d8d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -92,6 +92,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20c37ec03f264069"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02e0e55993bf441a"/>
 </x:worksheet>
 </file>
</xml_diff>